<commit_message>
add valueset R301 R286 R74 (#163) 9f03df294b8445a2050c2394a5f27ddb22a248e5
</commit_message>
<xml_diff>
--- a/ig/main/StructureDefinition-as-dp-organization.xlsx
+++ b/ig/main/StructureDefinition-as-dp-organization.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7761" uniqueCount="776">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7762" uniqueCount="776">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-01-11T15:09:13+00:00</t>
+    <t>2024-02-05T18:22:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -20980,7 +20980,7 @@
         <v>584</v>
       </c>
       <c r="D178" t="s" s="2">
-        <v>73</v>
+        <v>101</v>
       </c>
       <c r="E178" s="2"/>
       <c r="F178" t="s" s="2">
@@ -21007,7 +21007,9 @@
       <c r="M178" t="s" s="2">
         <v>191</v>
       </c>
-      <c r="N178" s="2"/>
+      <c r="N178" t="s" s="2">
+        <v>105</v>
+      </c>
       <c r="O178" s="2"/>
       <c r="P178" t="s" s="2">
         <v>73</v>

</xml_diff>